<commit_message>
Change name of Authorization extension (rm HealthcareService) (#211)
* change name authorization

* update hs

* Update AsAuthorizationExtension.fsh 76c012a280d4ed8b2dca521ffc68bbd283530eae
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-device.xlsx
+++ b/main/ig/StructureDefinition-as-device.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-06-05T12:07:44+00:00</t>
+    <t>2024-06-07T15:57:22+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -622,20 +622,20 @@
     <t>DomainResource.extension</t>
   </si>
   <si>
-    <t>Device.extension:as-ext-healthcareservice-authorization</t>
-  </si>
-  <si>
-    <t>as-ext-healthcareservice-authorization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-ext-healthcareservice-authorization}
+    <t>Device.extension:as-ext-authorization</t>
+  </si>
+  <si>
+    <t>as-ext-authorization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-ext-authorization}
 </t>
   </si>
   <si>
-    <t>AS HealthcareService Autorization Extension</t>
-  </si>
-  <si>
-    <t>Extension créée dans le cadre de l'Annuaire Santé pour décrire les autorisations  des activités sanitaires, sociales, médico-sociales et d'enseignement et des équipements matériels lourds autorisés.</t>
+    <t>AS Authorization Extension</t>
+  </si>
+  <si>
+    <t>Extension créée dans le cadre de l'Annuaire Santé pour décrire les autorisations des activités (HealthcareService) sanitaires, sociales, médico-sociales et d'enseignement et des équipements matériels (Device) lourds autorisés.</t>
   </si>
   <si>
     <t>Device.modifierExtension</t>
@@ -1908,9 +1908,9 @@
   <dimension ref="A1:AM86"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="53.01171875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="47.92578125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="37.6015625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="36.5703125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="22.67578125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="39.953125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="6.77734375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.9453125" customWidth="true" bestFit="true"/>

</xml_diff>